<commit_message>
adds summary section for tagged entries
</commit_message>
<xml_diff>
--- a/spec/data/time_log.xlsx
+++ b/spec/data/time_log.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="31">
   <si>
     <t xml:space="preserve">date</t>
   </si>
@@ -56,6 +56,9 @@
   </si>
   <si>
     <t xml:space="preserve">setup git repository</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ai</t>
   </si>
   <si>
     <t xml:space="preserve">dev</t>
@@ -126,6 +129,7 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -147,6 +151,7 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -191,40 +196,44 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -248,37 +257,37 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="000000"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="18a303"/>
+        <a:srgbClr val="18A303"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="0369a3"/>
+        <a:srgbClr val="0369A3"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="a33e03"/>
+        <a:srgbClr val="A33E03"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8e03a3"/>
+        <a:srgbClr val="8E03A3"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="c99c00"/>
+        <a:srgbClr val="C99C00"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="c9211e"/>
+        <a:srgbClr val="C9211E"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ee"/>
+        <a:srgbClr val="0000EE"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="551a8b"/>
+        <a:srgbClr val="551A8B"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
@@ -354,295 +363,303 @@
   <dimension ref="A1:G16"/>
   <sheetFormatPr defaultColWidth="11.515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="20.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="44.9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="20.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="44.9"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="4" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="5" t="n">
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="6" t="n">
         <v>42948</v>
       </c>
-      <c r="B2" s="6" t="n">
+      <c r="B2" s="7" t="n">
         <v>0.479166666666667</v>
       </c>
-      <c r="C2" s="6"/>
-      <c r="D2" s="7" t="s">
+      <c r="C2" s="7"/>
+      <c r="D2" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="E2" s="7" t="s">
+      <c r="E2" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="F2" s="8" t="s">
+      <c r="F2" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="G2" s="7"/>
-    </row>
-    <row r="3" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="5"/>
-      <c r="B3" s="6" t="n">
+      <c r="G2" s="8"/>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="6"/>
+      <c r="B3" s="7" t="n">
         <v>0.495138888888889</v>
       </c>
-      <c r="C3" s="6" t="n">
+      <c r="C3" s="7" t="n">
         <v>0.555555555555556</v>
       </c>
-      <c r="D3" s="7"/>
-      <c r="E3" s="7" t="s">
+      <c r="D3" s="8"/>
+      <c r="E3" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="F3" s="8" t="s">
+      <c r="F3" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="G3" s="7"/>
-    </row>
-    <row r="4" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="5"/>
-      <c r="B4" s="6" t="n">
+      <c r="G3" s="8" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="6"/>
+      <c r="B4" s="7" t="n">
         <v>0.583333333333333</v>
       </c>
-      <c r="C4" s="7"/>
-      <c r="D4" s="7"/>
-      <c r="E4" s="7" t="s">
+      <c r="C4" s="8"/>
+      <c r="D4" s="8"/>
+      <c r="E4" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="F4" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="G4" s="8"/>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="6"/>
+      <c r="B5" s="7" t="n">
+        <v>0.6875</v>
+      </c>
+      <c r="C5" s="7" t="n">
+        <v>0.791666666666667</v>
+      </c>
+      <c r="D5" s="8"/>
+      <c r="E5" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="F5" s="9"/>
+      <c r="G5" s="8"/>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="6"/>
+      <c r="B6" s="7" t="n">
+        <v>0.9375</v>
+      </c>
+      <c r="C6" s="7" t="n">
+        <v>0.979166666666667</v>
+      </c>
+      <c r="D6" s="8"/>
+      <c r="E6" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="F6" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="G6" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="F4" s="8" t="s">
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="6" t="n">
+        <v>42949</v>
+      </c>
+      <c r="B7" s="7" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="C7" s="7"/>
+      <c r="D7" s="8"/>
+      <c r="E7" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="G4" s="7"/>
-    </row>
-    <row r="5" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5"/>
-      <c r="B5" s="6" t="n">
-        <v>0.6875</v>
-      </c>
-      <c r="C5" s="6" t="n">
-        <v>0.791666666666667</v>
-      </c>
-      <c r="D5" s="7"/>
-      <c r="E5" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="F5" s="8"/>
-      <c r="G5" s="7"/>
-    </row>
-    <row r="6" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5"/>
-      <c r="B6" s="6" t="n">
-        <v>0.9375</v>
-      </c>
-      <c r="C6" s="6" t="n">
-        <v>0.979166666666667</v>
-      </c>
-      <c r="D6" s="7"/>
-      <c r="E6" s="7" t="s">
+      <c r="F7" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="G7" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="F6" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="G6" s="7"/>
-    </row>
-    <row r="7" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5" t="n">
-        <v>42949</v>
-      </c>
-      <c r="B7" s="6" t="n">
-        <v>0.35</v>
-      </c>
-      <c r="C7" s="6"/>
-      <c r="D7" s="7"/>
-      <c r="E7" s="7" t="s">
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="6"/>
+      <c r="B8" s="7" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="C8" s="7"/>
+      <c r="D8" s="8"/>
+      <c r="E8" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="F8" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="G8" s="8"/>
+    </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="6"/>
+      <c r="B9" s="7" t="n">
+        <v>0.40625</v>
+      </c>
+      <c r="C9" s="7" t="n">
+        <v>0.423611111111111</v>
+      </c>
+      <c r="D9" s="8"/>
+      <c r="E9" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="F9" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="G9" s="8"/>
+    </row>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="6"/>
+      <c r="B10" s="7" t="n">
+        <v>0.475694444444444</v>
+      </c>
+      <c r="C10" s="7" t="n">
+        <v>0.51875</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="E10" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="F10" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="G10" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="F7" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="G7" s="7"/>
-    </row>
-    <row r="8" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5"/>
-      <c r="B8" s="6" t="n">
-        <v>0.375</v>
-      </c>
-      <c r="C8" s="6"/>
-      <c r="D8" s="7"/>
-      <c r="E8" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="F8" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="G8" s="7"/>
-    </row>
-    <row r="9" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="5"/>
-      <c r="B9" s="6" t="n">
-        <v>0.40625</v>
-      </c>
-      <c r="C9" s="6" t="n">
-        <v>0.423611111111111</v>
-      </c>
-      <c r="D9" s="7"/>
-      <c r="E9" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="F9" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="G9" s="7"/>
-    </row>
-    <row r="10" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="5"/>
-      <c r="B10" s="6" t="n">
-        <v>0.475694444444444</v>
-      </c>
-      <c r="C10" s="6" t="n">
-        <v>0.51875</v>
-      </c>
-      <c r="D10" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="E10" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="F10" s="8" t="s">
+    </row>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="6"/>
+      <c r="B11" s="7" t="n">
+        <v>0.543055555555556</v>
+      </c>
+      <c r="C11" s="7" t="n">
+        <v>0.565277777777778</v>
+      </c>
+      <c r="D11" s="8"/>
+      <c r="E11" s="8"/>
+      <c r="F11" s="9"/>
+      <c r="G11" s="8"/>
+    </row>
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="6" t="n">
+        <v>42950</v>
+      </c>
+      <c r="B12" s="7" t="n">
+        <v>0.7125</v>
+      </c>
+      <c r="C12" s="7" t="n">
+        <v>0.811805555555556</v>
+      </c>
+      <c r="D12" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="E12" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="F12" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="G12" s="8"/>
+    </row>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="6"/>
+      <c r="B13" s="7" t="n">
+        <v>0.832638888888889</v>
+      </c>
+      <c r="C13" s="7"/>
+      <c r="D13" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="E13" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="F13" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="G13" s="8"/>
+    </row>
+    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="6"/>
+      <c r="B14" s="7" t="n">
+        <v>0.841666666666667</v>
+      </c>
+      <c r="C14" s="7"/>
+      <c r="D14" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="G10" s="7"/>
-    </row>
-    <row r="11" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="5"/>
-      <c r="B11" s="6" t="n">
-        <v>0.543055555555556</v>
-      </c>
-      <c r="C11" s="6" t="n">
-        <v>0.565277777777778</v>
-      </c>
-      <c r="D11" s="7"/>
-      <c r="E11" s="7"/>
-      <c r="F11" s="8"/>
-      <c r="G11" s="7"/>
-    </row>
-    <row r="12" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="5" t="n">
-        <v>42950</v>
-      </c>
-      <c r="B12" s="6" t="n">
-        <v>0.7125</v>
-      </c>
-      <c r="C12" s="6" t="n">
-        <v>0.811805555555556</v>
-      </c>
-      <c r="D12" s="7" t="s">
+      <c r="E14" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="F14" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="G14" s="8"/>
+    </row>
+    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="6"/>
+      <c r="B15" s="7" t="n">
+        <v>0.857638888888889</v>
+      </c>
+      <c r="C15" s="7"/>
+      <c r="D15" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="E15" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="F15" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="G15" s="8"/>
+    </row>
+    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="6"/>
+      <c r="B16" s="7" t="n">
+        <v>0.913888888888889</v>
+      </c>
+      <c r="C16" s="7" t="n">
+        <v>0.999305555555556</v>
+      </c>
+      <c r="D16" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="E12" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="F12" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="G12" s="7"/>
-    </row>
-    <row r="13" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="5"/>
-      <c r="B13" s="6" t="n">
-        <v>0.832638888888889</v>
-      </c>
-      <c r="C13" s="6"/>
-      <c r="D13" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="E13" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="F13" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="G13" s="7"/>
-    </row>
-    <row r="14" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="5"/>
-      <c r="B14" s="6" t="n">
-        <v>0.841666666666667</v>
-      </c>
-      <c r="C14" s="6"/>
-      <c r="D14" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="E14" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="F14" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="G14" s="7"/>
-    </row>
-    <row r="15" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="5"/>
-      <c r="B15" s="6" t="n">
-        <v>0.857638888888889</v>
-      </c>
-      <c r="C15" s="6"/>
-      <c r="D15" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="E15" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="F15" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="G15" s="7"/>
-    </row>
-    <row r="16" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="5"/>
-      <c r="B16" s="6" t="n">
-        <v>0.913888888888889</v>
-      </c>
-      <c r="C16" s="6" t="n">
-        <v>0.999305555555556</v>
-      </c>
-      <c r="D16" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="E16" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="F16" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="G16" s="7"/>
+      <c r="E16" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="F16" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="G16" s="8"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
+    <oddHeader>&amp;C&amp;"Times New Roman"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman"&amp;12Page &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
</xml_diff>